<commit_message>
admin updates and subscription
</commit_message>
<xml_diff>
--- a/Vrindhavanam Glassmorphism/Vrindhavanam/cardamom.xlsx
+++ b/Vrindhavanam Glassmorphism/Vrindhavanam/cardamom.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Glassmorphism\Vrindavanam Glassmorphism\Vrindavanam\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Glassmorphism\Vrindhavanam Glassmorphism\Vrindhavanam\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04189A32-F57E-4DA9-946D-C820FBFB5BD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7570CB66-9588-4FB7-B566-65B265CE2337}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{213A37A3-F88C-42DF-B134-BBBC12CBE028}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{213A37A3-F88C-42DF-B134-BBBC12CBE028}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="509" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="78">
   <si>
     <t>Cardamom</t>
   </si>
@@ -265,6 +265,9 @@
   </si>
   <si>
     <t xml:space="preserve">Organic </t>
+  </si>
+  <si>
+    <t>stock_quantity</t>
   </si>
 </sst>
 </file>
@@ -623,7 +626,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0EDA5FEE-3D0D-4201-B43F-EBBD6EEA5F86}">
-  <dimension ref="A1:N58"/>
+  <dimension ref="A1:O58"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.6640625" customWidth="1"/>
@@ -640,9 +643,10 @@
     <col min="12" max="12" width="16.88671875" customWidth="1"/>
     <col min="13" max="13" width="21.33203125" customWidth="1"/>
     <col min="14" max="14" width="16.5546875" customWidth="1"/>
+    <col min="15" max="15" width="17.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>48</v>
       </c>
@@ -685,8 +689,11 @@
       <c r="N1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -729,8 +736,11 @@
       <c r="N2">
         <v>1500</v>
       </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -773,8 +783,11 @@
       <c r="N3">
         <v>2000</v>
       </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -817,8 +830,11 @@
       <c r="N4">
         <v>3000</v>
       </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -861,8 +877,11 @@
       <c r="N5">
         <v>5600</v>
       </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O5">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -905,8 +924,11 @@
       <c r="N6">
         <v>9000</v>
       </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O6">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -949,8 +971,11 @@
       <c r="N7">
         <v>200</v>
       </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -993,8 +1018,11 @@
       <c r="N8">
         <v>800</v>
       </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1037,8 +1065,11 @@
       <c r="N9">
         <v>1500</v>
       </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O9">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1081,8 +1112,11 @@
       <c r="N10">
         <v>2000</v>
       </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O10">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1125,8 +1159,11 @@
       <c r="N11">
         <v>2500</v>
       </c>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1169,8 +1206,11 @@
       <c r="N12">
         <v>100</v>
       </c>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O12">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1213,8 +1253,11 @@
       <c r="N13">
         <v>400</v>
       </c>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O13">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1257,8 +1300,11 @@
       <c r="N14">
         <v>900</v>
       </c>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O14">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1301,8 +1347,11 @@
       <c r="N15">
         <v>2000</v>
       </c>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O15">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1345,8 +1394,11 @@
       <c r="N16">
         <v>2500</v>
       </c>
-    </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O16">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1389,8 +1441,11 @@
       <c r="N17">
         <v>200</v>
       </c>
-    </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O17">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1433,8 +1488,11 @@
       <c r="N18">
         <v>600</v>
       </c>
-    </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O18">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1477,8 +1535,11 @@
       <c r="N19">
         <v>1200</v>
       </c>
-    </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O19">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1521,8 +1582,11 @@
       <c r="N20">
         <v>2000</v>
       </c>
-    </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O20">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1565,8 +1629,11 @@
       <c r="N21">
         <v>2500</v>
       </c>
-    </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O21">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1609,8 +1676,11 @@
       <c r="N22">
         <v>200</v>
       </c>
-    </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O22">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1653,8 +1723,11 @@
       <c r="N23">
         <v>600</v>
       </c>
-    </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O23">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1697,8 +1770,11 @@
       <c r="N24">
         <v>900</v>
       </c>
-    </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O24">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1741,8 +1817,11 @@
       <c r="N25">
         <v>1600</v>
       </c>
-    </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O25">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1785,8 +1864,11 @@
       <c r="N26">
         <v>2000</v>
       </c>
-    </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O26">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1829,8 +1911,11 @@
       <c r="N27">
         <v>200</v>
       </c>
-    </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O27">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1873,8 +1958,11 @@
       <c r="N28">
         <v>600</v>
       </c>
-    </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O28">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1917,8 +2005,11 @@
       <c r="N29">
         <v>900</v>
       </c>
-    </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O29">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1961,8 +2052,11 @@
       <c r="N30">
         <v>1600</v>
       </c>
-    </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O30">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>30</v>
       </c>
@@ -2005,8 +2099,11 @@
       <c r="N31">
         <v>2000</v>
       </c>
-    </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O31">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>31</v>
       </c>
@@ -2049,8 +2146,11 @@
       <c r="N32">
         <v>200</v>
       </c>
-    </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O32">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="33" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>32</v>
       </c>
@@ -2093,8 +2193,11 @@
       <c r="N33">
         <v>600</v>
       </c>
-    </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O33">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="34" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>33</v>
       </c>
@@ -2137,8 +2240,11 @@
       <c r="N34">
         <v>900</v>
       </c>
-    </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O34">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="35" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>34</v>
       </c>
@@ -2181,8 +2287,11 @@
       <c r="N35">
         <v>1600</v>
       </c>
-    </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O35">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="36" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>35</v>
       </c>
@@ -2225,8 +2334,11 @@
       <c r="N36">
         <v>2000</v>
       </c>
-    </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O36">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="37" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>36</v>
       </c>
@@ -2269,8 +2381,11 @@
       <c r="N37">
         <v>200</v>
       </c>
-    </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O37">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="38" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>37</v>
       </c>
@@ -2313,8 +2428,11 @@
       <c r="N38">
         <v>600</v>
       </c>
-    </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O38">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="39" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>38</v>
       </c>
@@ -2357,8 +2475,11 @@
       <c r="N39">
         <v>900</v>
       </c>
-    </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O39">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="40" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>39</v>
       </c>
@@ -2401,8 +2522,11 @@
       <c r="N40">
         <v>1600</v>
       </c>
-    </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O40">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="41" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>40</v>
       </c>
@@ -2445,8 +2569,11 @@
       <c r="N41">
         <v>2000</v>
       </c>
-    </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O41">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="42" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>41</v>
       </c>
@@ -2489,8 +2616,11 @@
       <c r="N42">
         <v>200</v>
       </c>
-    </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O42">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>42</v>
       </c>
@@ -2533,8 +2663,11 @@
       <c r="N43">
         <v>600</v>
       </c>
-    </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O43">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>43</v>
       </c>
@@ -2577,8 +2710,11 @@
       <c r="N44">
         <v>900</v>
       </c>
-    </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O44">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="45" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>44</v>
       </c>
@@ -2621,8 +2757,11 @@
       <c r="N45">
         <v>1600</v>
       </c>
-    </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O45">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="46" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>45</v>
       </c>
@@ -2665,8 +2804,11 @@
       <c r="N46">
         <v>2000</v>
       </c>
-    </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O46">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="47" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>46</v>
       </c>
@@ -2709,8 +2851,11 @@
       <c r="N47">
         <v>200</v>
       </c>
-    </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O47">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="48" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>47</v>
       </c>
@@ -2753,8 +2898,11 @@
       <c r="N48">
         <v>600</v>
       </c>
-    </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O48">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="49" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>48</v>
       </c>
@@ -2797,8 +2945,11 @@
       <c r="N49">
         <v>900</v>
       </c>
-    </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O49">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="50" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>49</v>
       </c>
@@ -2841,8 +2992,11 @@
       <c r="N50">
         <v>1600</v>
       </c>
-    </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O50">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="51" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>50</v>
       </c>
@@ -2885,8 +3039,11 @@
       <c r="N51">
         <v>2000</v>
       </c>
-    </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O51">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="52" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>51</v>
       </c>
@@ -2929,8 +3086,11 @@
       <c r="N52">
         <v>200</v>
       </c>
-    </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O52">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="53" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>52</v>
       </c>
@@ -2973,8 +3133,11 @@
       <c r="N53">
         <v>600</v>
       </c>
-    </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O53">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="54" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>53</v>
       </c>
@@ -3017,8 +3180,11 @@
       <c r="N54">
         <v>900</v>
       </c>
-    </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O54">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="55" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>54</v>
       </c>
@@ -3061,8 +3227,11 @@
       <c r="N55">
         <v>1600</v>
       </c>
-    </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O55">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="56" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>55</v>
       </c>
@@ -3105,11 +3274,14 @@
       <c r="N56">
         <v>2000</v>
       </c>
-    </row>
-    <row r="57" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O56">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="57" spans="1:15" x14ac:dyDescent="0.3">
       <c r="H57" s="1"/>
     </row>
-    <row r="58" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:15" x14ac:dyDescent="0.3">
       <c r="H58" s="1"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remove node_modules from repository
</commit_message>
<xml_diff>
--- a/Vrindhavanam Glassmorphism/Vrindhavanam/cardamom.xlsx
+++ b/Vrindhavanam Glassmorphism/Vrindhavanam/cardamom.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Glassmorphism\Vrindhavanam Glassmorphism\Vrindhavanam\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Glassmorphism\Vrindavanam Glassmorphism\Vrindavanam\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7570CB66-9588-4FB7-B566-65B265CE2337}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04189A32-F57E-4DA9-946D-C820FBFB5BD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{213A37A3-F88C-42DF-B134-BBBC12CBE028}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{213A37A3-F88C-42DF-B134-BBBC12CBE028}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="509" uniqueCount="77">
   <si>
     <t>Cardamom</t>
   </si>
@@ -265,9 +265,6 @@
   </si>
   <si>
     <t xml:space="preserve">Organic </t>
-  </si>
-  <si>
-    <t>stock_quantity</t>
   </si>
 </sst>
 </file>
@@ -626,7 +623,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0EDA5FEE-3D0D-4201-B43F-EBBD6EEA5F86}">
-  <dimension ref="A1:O58"/>
+  <dimension ref="A1:N58"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.6640625" customWidth="1"/>
@@ -643,10 +640,9 @@
     <col min="12" max="12" width="16.88671875" customWidth="1"/>
     <col min="13" max="13" width="21.33203125" customWidth="1"/>
     <col min="14" max="14" width="16.5546875" customWidth="1"/>
-    <col min="15" max="15" width="17.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>48</v>
       </c>
@@ -689,11 +685,8 @@
       <c r="N1" t="s">
         <v>11</v>
       </c>
-      <c r="O1" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -736,11 +729,8 @@
       <c r="N2">
         <v>1500</v>
       </c>
-      <c r="O2">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -783,11 +773,8 @@
       <c r="N3">
         <v>2000</v>
       </c>
-      <c r="O3">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -830,11 +817,8 @@
       <c r="N4">
         <v>3000</v>
       </c>
-      <c r="O4">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -877,11 +861,8 @@
       <c r="N5">
         <v>5600</v>
       </c>
-      <c r="O5">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -924,11 +905,8 @@
       <c r="N6">
         <v>9000</v>
       </c>
-      <c r="O6">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -971,11 +949,8 @@
       <c r="N7">
         <v>200</v>
       </c>
-      <c r="O7">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1018,11 +993,8 @@
       <c r="N8">
         <v>800</v>
       </c>
-      <c r="O8">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1065,11 +1037,8 @@
       <c r="N9">
         <v>1500</v>
       </c>
-      <c r="O9">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1112,11 +1081,8 @@
       <c r="N10">
         <v>2000</v>
       </c>
-      <c r="O10">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1159,11 +1125,8 @@
       <c r="N11">
         <v>2500</v>
       </c>
-      <c r="O11">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1206,11 +1169,8 @@
       <c r="N12">
         <v>100</v>
       </c>
-      <c r="O12">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1253,11 +1213,8 @@
       <c r="N13">
         <v>400</v>
       </c>
-      <c r="O13">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1300,11 +1257,8 @@
       <c r="N14">
         <v>900</v>
       </c>
-      <c r="O14">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1347,11 +1301,8 @@
       <c r="N15">
         <v>2000</v>
       </c>
-      <c r="O15">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1394,11 +1345,8 @@
       <c r="N16">
         <v>2500</v>
       </c>
-      <c r="O16">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1441,11 +1389,8 @@
       <c r="N17">
         <v>200</v>
       </c>
-      <c r="O17">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1488,11 +1433,8 @@
       <c r="N18">
         <v>600</v>
       </c>
-      <c r="O18">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1535,11 +1477,8 @@
       <c r="N19">
         <v>1200</v>
       </c>
-      <c r="O19">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1582,11 +1521,8 @@
       <c r="N20">
         <v>2000</v>
       </c>
-      <c r="O20">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1629,11 +1565,8 @@
       <c r="N21">
         <v>2500</v>
       </c>
-      <c r="O21">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1676,11 +1609,8 @@
       <c r="N22">
         <v>200</v>
       </c>
-      <c r="O22">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1723,11 +1653,8 @@
       <c r="N23">
         <v>600</v>
       </c>
-      <c r="O23">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1770,11 +1697,8 @@
       <c r="N24">
         <v>900</v>
       </c>
-      <c r="O24">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1817,11 +1741,8 @@
       <c r="N25">
         <v>1600</v>
       </c>
-      <c r="O25">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1864,11 +1785,8 @@
       <c r="N26">
         <v>2000</v>
       </c>
-      <c r="O26">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1911,11 +1829,8 @@
       <c r="N27">
         <v>200</v>
       </c>
-      <c r="O27">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1958,11 +1873,8 @@
       <c r="N28">
         <v>600</v>
       </c>
-      <c r="O28">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>28</v>
       </c>
@@ -2005,11 +1917,8 @@
       <c r="N29">
         <v>900</v>
       </c>
-      <c r="O29">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>29</v>
       </c>
@@ -2052,11 +1961,8 @@
       <c r="N30">
         <v>1600</v>
       </c>
-      <c r="O30">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>30</v>
       </c>
@@ -2099,11 +2005,8 @@
       <c r="N31">
         <v>2000</v>
       </c>
-      <c r="O31">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>31</v>
       </c>
@@ -2146,11 +2049,8 @@
       <c r="N32">
         <v>200</v>
       </c>
-      <c r="O32">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>32</v>
       </c>
@@ -2193,11 +2093,8 @@
       <c r="N33">
         <v>600</v>
       </c>
-      <c r="O33">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>33</v>
       </c>
@@ -2240,11 +2137,8 @@
       <c r="N34">
         <v>900</v>
       </c>
-      <c r="O34">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>34</v>
       </c>
@@ -2287,11 +2181,8 @@
       <c r="N35">
         <v>1600</v>
       </c>
-      <c r="O35">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>35</v>
       </c>
@@ -2334,11 +2225,8 @@
       <c r="N36">
         <v>2000</v>
       </c>
-      <c r="O36">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>36</v>
       </c>
@@ -2381,11 +2269,8 @@
       <c r="N37">
         <v>200</v>
       </c>
-      <c r="O37">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>37</v>
       </c>
@@ -2428,11 +2313,8 @@
       <c r="N38">
         <v>600</v>
       </c>
-      <c r="O38">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="39" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>38</v>
       </c>
@@ -2475,11 +2357,8 @@
       <c r="N39">
         <v>900</v>
       </c>
-      <c r="O39">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>39</v>
       </c>
@@ -2522,11 +2401,8 @@
       <c r="N40">
         <v>1600</v>
       </c>
-      <c r="O40">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="41" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>40</v>
       </c>
@@ -2569,11 +2445,8 @@
       <c r="N41">
         <v>2000</v>
       </c>
-      <c r="O41">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="42" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>41</v>
       </c>
@@ -2616,11 +2489,8 @@
       <c r="N42">
         <v>200</v>
       </c>
-      <c r="O42">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="43" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>42</v>
       </c>
@@ -2663,11 +2533,8 @@
       <c r="N43">
         <v>600</v>
       </c>
-      <c r="O43">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="44" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>43</v>
       </c>
@@ -2710,11 +2577,8 @@
       <c r="N44">
         <v>900</v>
       </c>
-      <c r="O44">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>44</v>
       </c>
@@ -2757,11 +2621,8 @@
       <c r="N45">
         <v>1600</v>
       </c>
-      <c r="O45">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>45</v>
       </c>
@@ -2804,11 +2665,8 @@
       <c r="N46">
         <v>2000</v>
       </c>
-      <c r="O46">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>46</v>
       </c>
@@ -2851,11 +2709,8 @@
       <c r="N47">
         <v>200</v>
       </c>
-      <c r="O47">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>47</v>
       </c>
@@ -2898,11 +2753,8 @@
       <c r="N48">
         <v>600</v>
       </c>
-      <c r="O48">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="49" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>48</v>
       </c>
@@ -2945,11 +2797,8 @@
       <c r="N49">
         <v>900</v>
       </c>
-      <c r="O49">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="50" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>49</v>
       </c>
@@ -2992,11 +2841,8 @@
       <c r="N50">
         <v>1600</v>
       </c>
-      <c r="O50">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="51" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>50</v>
       </c>
@@ -3039,11 +2885,8 @@
       <c r="N51">
         <v>2000</v>
       </c>
-      <c r="O51">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="52" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>51</v>
       </c>
@@ -3086,11 +2929,8 @@
       <c r="N52">
         <v>200</v>
       </c>
-      <c r="O52">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="53" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>52</v>
       </c>
@@ -3133,11 +2973,8 @@
       <c r="N53">
         <v>600</v>
       </c>
-      <c r="O53">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="54" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>53</v>
       </c>
@@ -3180,11 +3017,8 @@
       <c r="N54">
         <v>900</v>
       </c>
-      <c r="O54">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="55" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>54</v>
       </c>
@@ -3227,11 +3061,8 @@
       <c r="N55">
         <v>1600</v>
       </c>
-      <c r="O55">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="56" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>55</v>
       </c>
@@ -3274,14 +3105,11 @@
       <c r="N56">
         <v>2000</v>
       </c>
-      <c r="O56">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="57" spans="1:14" x14ac:dyDescent="0.3">
       <c r="H57" s="1"/>
     </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:14" x14ac:dyDescent="0.3">
       <c r="H58" s="1"/>
     </row>
   </sheetData>

</xml_diff>